<commit_message>
Update March 30 rp
</commit_message>
<xml_diff>
--- a/data/Mar/10-03-2026/NGAY 10-3.xlsx
+++ b/data/Mar/10-03-2026/NGAY 10-3.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\TextExtractorTool\data\Mar\10-03-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Mar\10-03-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28ACEC0D-C117-4F9A-99A2-4CD493652BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434DCDDC-3466-422E-A592-29E8E60E3FB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{71C05EAB-372E-4558-9B67-2A0333D33C4F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{71C05EAB-372E-4558-9B67-2A0333D33C4F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$Q$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$Q$64</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="168">
   <si>
     <t>Tình trạng TT</t>
   </si>
@@ -480,15 +480,6 @@
     <t>09-03-2026</t>
   </si>
   <si>
-    <t>Phẩm Huỳnh</t>
-  </si>
-  <si>
-    <t>HD136278</t>
-  </si>
-  <si>
-    <t>84 phạm Hồng thái phường bến thành</t>
-  </si>
-  <si>
     <t>parichat jaiduang</t>
   </si>
   <si>
@@ -496,15 +487,6 @@
   </si>
   <si>
     <t>Central 2 Building (C2), Vinhomes Central Park, 208 Nguyen H</t>
-  </si>
-  <si>
-    <t>Lê Thị Mỹ Quyên</t>
-  </si>
-  <si>
-    <t>HD136315</t>
-  </si>
-  <si>
-    <t>Địa chỉ: 334 tô hiến thành p14 Chung cư kingdom block A</t>
   </si>
   <si>
     <t>W3136</t>
@@ -1242,7 +1224,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F28604F7-D21B-4533-8AD0-8E4BB48433FE}">
-  <dimension ref="A1:Q75"/>
+  <dimension ref="A1:Q73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -2445,11 +2427,11 @@
         <v>845</v>
       </c>
       <c r="H31" s="30">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I31" s="30">
         <f t="shared" si="0"/>
-        <v>820</v>
+        <v>845</v>
       </c>
       <c r="J31" t="s">
         <v>16</v>
@@ -2486,18 +2468,18 @@
       <c r="E32" t="s">
         <v>149</v>
       </c>
-      <c r="F32" s="29">
-        <v>1</v>
+      <c r="F32" s="29" t="s">
+        <v>19</v>
       </c>
       <c r="G32" s="30">
+        <v>2600</v>
+      </c>
+      <c r="H32" s="30">
         <v>0</v>
       </c>
-      <c r="H32" s="30">
-        <v>25</v>
-      </c>
       <c r="I32" s="30">
-        <f>-H32</f>
-        <v>-25</v>
+        <f>G32-H32</f>
+        <v>2600</v>
       </c>
       <c r="J32" t="s">
         <v>16</v>
@@ -2534,36 +2516,27 @@
       <c r="E33" t="s">
         <v>152</v>
       </c>
-      <c r="F33" s="29" t="s">
-        <v>19</v>
+      <c r="F33" s="29">
+        <v>12</v>
       </c>
       <c r="G33" s="30">
-        <v>2600</v>
+        <v>0</v>
       </c>
       <c r="H33" s="30">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I33" s="30">
-        <f>G33-H33</f>
-        <v>2575</v>
+        <f>-H33</f>
+        <v>-30</v>
       </c>
       <c r="J33" t="s">
-        <v>16</v>
+        <v>61</v>
       </c>
       <c r="K33" t="s">
         <v>23</v>
       </c>
       <c r="L33" t="s">
-        <v>146</v>
-      </c>
-      <c r="M33" t="s">
-        <v>39</v>
-      </c>
-      <c r="N33" t="s">
-        <v>17</v>
-      </c>
-      <c r="P33" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="Q33">
         <v>1</v>
@@ -2583,68 +2556,59 @@
         <v>155</v>
       </c>
       <c r="F34" s="29">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G34" s="30">
-        <v>25</v>
+        <v>850</v>
       </c>
       <c r="H34" s="30">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="I34" s="30">
         <f>G34-H34</f>
-        <v>0</v>
+        <v>820</v>
       </c>
       <c r="J34" t="s">
-        <v>16</v>
+        <v>61</v>
       </c>
       <c r="K34" t="s">
         <v>23</v>
       </c>
       <c r="L34" t="s">
-        <v>146</v>
-      </c>
-      <c r="M34" t="s">
-        <v>39</v>
-      </c>
-      <c r="N34" t="s">
-        <v>17</v>
-      </c>
-      <c r="P34" t="s">
-        <v>18</v>
+        <v>57</v>
       </c>
       <c r="Q34">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>156</v>
+      </c>
       <c r="B35" t="s">
         <v>52</v>
       </c>
       <c r="C35" t="s">
-        <v>156</v>
-      </c>
-      <c r="D35" t="s">
         <v>157</v>
       </c>
       <c r="E35" t="s">
         <v>158</v>
       </c>
       <c r="F35" s="29">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G35" s="30">
-        <v>0</v>
+        <v>1065</v>
       </c>
       <c r="H35" s="30">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="I35" s="30">
-        <f>-H35</f>
-        <v>-30</v>
+        <f>G35-H35</f>
+        <v>1030</v>
       </c>
       <c r="J35" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="K35" t="s">
         <v>23</v>
@@ -2657,39 +2621,42 @@
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>156</v>
+      </c>
       <c r="B36" t="s">
         <v>52</v>
       </c>
       <c r="C36" t="s">
         <v>159</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
         <v>160</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" s="29">
+        <v>4</v>
+      </c>
+      <c r="G36" s="30">
+        <v>0</v>
+      </c>
+      <c r="H36" s="30">
+        <v>25</v>
+      </c>
+      <c r="I36" s="30">
+        <f>-H36</f>
+        <v>-25</v>
+      </c>
+      <c r="J36" t="s">
+        <v>56</v>
+      </c>
+      <c r="K36" t="s">
+        <v>23</v>
+      </c>
+      <c r="L36" t="s">
+        <v>57</v>
+      </c>
+      <c r="M36" t="s">
         <v>161</v>
-      </c>
-      <c r="F36" s="29">
-        <v>9</v>
-      </c>
-      <c r="G36" s="30">
-        <v>850</v>
-      </c>
-      <c r="H36" s="30">
-        <v>30</v>
-      </c>
-      <c r="I36" s="30">
-        <f>G36-H36</f>
-        <v>820</v>
-      </c>
-      <c r="J36" t="s">
-        <v>61</v>
-      </c>
-      <c r="K36" t="s">
-        <v>23</v>
-      </c>
-      <c r="L36" t="s">
-        <v>57</v>
       </c>
       <c r="Q36">
         <v>1</v>
@@ -2697,38 +2664,41 @@
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>156</v>
+      </c>
+      <c r="B37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C37" t="s">
         <v>162</v>
       </c>
-      <c r="B37" t="s">
-        <v>52</v>
-      </c>
-      <c r="C37" t="s">
+      <c r="E37" t="s">
         <v>163</v>
       </c>
-      <c r="E37" t="s">
-        <v>164</v>
-      </c>
-      <c r="F37" s="29">
-        <v>9</v>
+      <c r="F37" s="29" t="s">
+        <v>15</v>
       </c>
       <c r="G37" s="30">
-        <v>1065</v>
+        <v>2170</v>
       </c>
       <c r="H37" s="30">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="I37" s="30">
         <f>G37-H37</f>
-        <v>1030</v>
+        <v>2140</v>
       </c>
       <c r="J37" t="s">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="K37" t="s">
         <v>23</v>
       </c>
       <c r="L37" t="s">
         <v>57</v>
+      </c>
+      <c r="M37" t="s">
+        <v>164</v>
       </c>
       <c r="Q37">
         <v>1</v>
@@ -2736,7 +2706,7 @@
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B38" t="s">
         <v>52</v>
@@ -2747,21 +2717,21 @@
       <c r="E38" t="s">
         <v>166</v>
       </c>
-      <c r="F38" s="29">
-        <v>4</v>
+      <c r="F38" s="29" t="s">
+        <v>15</v>
       </c>
       <c r="G38" s="30">
+        <v>30</v>
+      </c>
+      <c r="H38" s="30">
+        <v>30</v>
+      </c>
+      <c r="I38" s="30">
+        <f>G38-H38</f>
         <v>0</v>
       </c>
-      <c r="H38" s="30">
-        <v>25</v>
-      </c>
-      <c r="I38" s="30">
-        <f>-H38</f>
-        <v>-25</v>
-      </c>
       <c r="J38" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="K38" t="s">
         <v>23</v>
@@ -2770,232 +2740,214 @@
         <v>57</v>
       </c>
       <c r="M38" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="Q38">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>162</v>
-      </c>
-      <c r="B39" t="s">
-        <v>52</v>
-      </c>
-      <c r="C39" t="s">
-        <v>168</v>
-      </c>
-      <c r="E39" t="s">
-        <v>169</v>
-      </c>
-      <c r="F39" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="G39" s="30">
-        <v>2170</v>
-      </c>
-      <c r="H39" s="30">
-        <v>30</v>
-      </c>
-      <c r="I39" s="30">
-        <f>G39-H39</f>
-        <v>2140</v>
-      </c>
-      <c r="J39" t="s">
-        <v>23</v>
-      </c>
-      <c r="K39" t="s">
-        <v>23</v>
-      </c>
-      <c r="L39" t="s">
-        <v>57</v>
-      </c>
-      <c r="M39" t="s">
-        <v>170</v>
-      </c>
-      <c r="Q39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>162</v>
-      </c>
-      <c r="B40" t="s">
-        <v>52</v>
-      </c>
-      <c r="C40" t="s">
-        <v>171</v>
-      </c>
-      <c r="E40" t="s">
-        <v>172</v>
-      </c>
-      <c r="F40" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="G40" s="30">
-        <v>30</v>
-      </c>
-      <c r="H40" s="30">
-        <v>30</v>
-      </c>
-      <c r="I40" s="30">
-        <f>G40-H40</f>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="G41">
+        <f>SUBTOTAL(9,G3:G38)</f>
+        <v>23675</v>
+      </c>
+      <c r="H41">
+        <f>SUBTOTAL(9,H3:H38)</f>
+        <v>935</v>
+      </c>
+      <c r="I41">
+        <f>SUBTOTAL(9,I3:I38)</f>
+        <v>22740</v>
+      </c>
+      <c r="J41">
+        <f>SUBTOTAL(9,J3:J38)</f>
         <v>0</v>
       </c>
-      <c r="J40" t="s">
-        <v>23</v>
-      </c>
-      <c r="K40" t="s">
-        <v>23</v>
-      </c>
-      <c r="L40" t="s">
-        <v>57</v>
-      </c>
-      <c r="M40" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="G43">
-        <f t="shared" ref="G43:M43" si="1">SUBTOTAL(9,G3:G40)</f>
-        <v>23700</v>
-      </c>
-      <c r="H43">
-        <f t="shared" si="1"/>
-        <v>1035</v>
-      </c>
-      <c r="I43">
-        <f t="shared" si="1"/>
-        <v>22665</v>
-      </c>
-      <c r="J43">
+      <c r="K41">
+        <f>SUBTOTAL(9,K3:K38)</f>
+        <v>0</v>
+      </c>
+      <c r="L41">
+        <f>SUBTOTAL(9,L3:L38)</f>
+        <v>0</v>
+      </c>
+      <c r="M41">
+        <f>SUBTOTAL(9,M3:M38)</f>
+        <v>0</v>
+      </c>
+      <c r="N41">
+        <f t="shared" ref="N41:Q41" si="1">SUBTOTAL(9,N3:N38)</f>
+        <v>0</v>
+      </c>
+      <c r="O41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K43">
+      <c r="P41">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L43">
+      <c r="Q41">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M43">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N43">
-        <f t="shared" ref="N43:Q43" si="2">SUBTOTAL(9,N3:N40)</f>
-        <v>0</v>
-      </c>
-      <c r="O43">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P43">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q43">
-        <f t="shared" si="2"/>
-        <v>38</v>
-      </c>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B43" s="1"/>
+      <c r="C43" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="D43" s="45"/>
+      <c r="E43" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L43" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M43" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="N43" s="5"/>
+      <c r="O43" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="P43" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q43" s="5"/>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A44" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C44" s="46">
+        <f>SUMIFS(G$3:G$73,$B$3:$B$73,$A43,$L$3:$L$73,$A44)</f>
+        <v>20230</v>
+      </c>
+      <c r="D44" s="47"/>
+      <c r="E44" s="9">
+        <f>SUMIFS(Q$3:Q$73,$B$3:$B$73,$A43,$L$3:$L$73,$A44)</f>
+        <v>34</v>
+      </c>
+      <c r="F44" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="G44" s="5"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="K44" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="L44" s="12">
+        <f>SUMIFS(G$3:G$73,$J$3:$J$73,$K43)</f>
+        <v>1455</v>
+      </c>
+      <c r="M44" s="12">
+        <f>SUMIFS(Q3:Q73,J3:J73,K43)</f>
+        <v>2</v>
+      </c>
+      <c r="N44" s="5"/>
+      <c r="O44" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="P44" s="13">
+        <v>11243</v>
+      </c>
+      <c r="Q44" s="5"/>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B45" s="1"/>
-      <c r="C45" s="44" t="s">
-        <v>24</v>
-      </c>
-      <c r="D45" s="45"/>
-      <c r="E45" s="4" t="s">
-        <v>25</v>
+      <c r="A45" s="5"/>
+      <c r="B45" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="48">
+        <f>-SUMIFS(H$3:H$73,$B$3:$B$73,$A43,$L$3:$L$73,$A44)</f>
+        <v>-935</v>
+      </c>
+      <c r="D45" s="49"/>
+      <c r="E45" s="15">
+        <f>SUMIFS(Q$3:Q$73,$B$3:$B$73,$A43,$L$3:$L$73,$A44)</f>
+        <v>34</v>
       </c>
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
-      <c r="H45" s="6"/>
+      <c r="H45" s="5"/>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
-      <c r="K45" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="L45" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="M45" s="7" t="s">
-        <v>25</v>
-      </c>
+      <c r="K45" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="L45" s="12"/>
+      <c r="M45" s="16"/>
       <c r="N45" s="5"/>
-      <c r="O45" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="P45" s="8" t="s">
-        <v>173</v>
+      <c r="O45" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="P45" s="13">
+        <v>1345</v>
       </c>
       <c r="Q45" s="5"/>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A46" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C46" s="46">
-        <f>SUMIFS(G$3:G$75,$B$3:$B$75,$A45,$L$3:$L$75,$A46)</f>
-        <v>20230</v>
-      </c>
-      <c r="D46" s="47"/>
-      <c r="E46" s="9">
-        <f>SUMIFS(Q$3:Q$75,$B$3:$B$75,$A45,$L$3:$L$75,$A46)</f>
-        <v>34</v>
-      </c>
-      <c r="F46" s="10" t="s">
-        <v>29</v>
-      </c>
+      <c r="A46" s="5"/>
+      <c r="B46" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C46" s="50">
+        <f>-SUMIFS(I$3:I$68,$B$3:$B$68,$A43,$P$3:$P$68,"xx",$N$3:$N$68,"x")</f>
+        <v>-3445</v>
+      </c>
+      <c r="D46" s="51"/>
+      <c r="E46" s="17">
+        <f>SUMIFS($Q$3:$Q$77,$B$3:$B$77,$A43,$P$3:$P$77,"xx",$N$3:$N$77,"x")</f>
+        <v>2</v>
+      </c>
+      <c r="F46" s="5"/>
       <c r="G46" s="5"/>
-      <c r="H46" s="6"/>
+      <c r="H46" s="5"/>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
-      <c r="K46" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="L46" s="12">
-        <f>SUMIFS(G$3:G$75,$J$3:$J$75,$K45)</f>
-        <v>1455</v>
-      </c>
-      <c r="M46" s="12">
-        <f>SUMIFS(Q3:Q75,J3:J75,K45)</f>
-        <v>2</v>
-      </c>
+      <c r="K46" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="L46" s="19"/>
+      <c r="M46" s="16"/>
       <c r="N46" s="5"/>
       <c r="O46" s="13" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="P46" s="13">
-        <v>11243</v>
+        <v>14282</v>
       </c>
       <c r="Q46" s="5"/>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="5"/>
-      <c r="B47" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C47" s="48">
-        <f>-SUMIFS(H$3:H$75,$B$3:$B$75,$A45,$L$3:$L$75,$A46)</f>
-        <v>-935</v>
-      </c>
-      <c r="D47" s="49"/>
-      <c r="E47" s="15">
-        <f>SUMIFS(Q$3:Q$75,$B$3:$B$75,$A45,$L$3:$L$75,$A46)</f>
+      <c r="B47" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C47" s="52">
+        <f>SUBTOTAL(9,C43:C46)</f>
+        <v>15850</v>
+      </c>
+      <c r="D47" s="53"/>
+      <c r="E47" s="21">
+        <f>E44</f>
         <v>34</v>
       </c>
       <c r="F47" s="5"/>
@@ -3003,369 +2955,303 @@
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
-      <c r="K47" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="L47" s="12"/>
-      <c r="M47" s="16"/>
+      <c r="K47" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="L47" s="23"/>
+      <c r="M47" s="23"/>
       <c r="N47" s="5"/>
       <c r="O47" s="13" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="P47" s="13">
-        <v>1345</v>
+        <v>6005</v>
       </c>
       <c r="Q47" s="5"/>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="5"/>
-      <c r="B48" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C48" s="50">
-        <f>-SUMIFS(I$3:I$70,$B$3:$B$70,$A45,$P$3:$P$70,"xx",$N$3:$N$70,"x")</f>
-        <v>-3370</v>
-      </c>
-      <c r="D48" s="51"/>
-      <c r="E48" s="17">
-        <f>SUMIFS($Q$3:$Q$79,$B$3:$B$79,$A45,$P$3:$P$79,"xx",$N$3:$N$79,"x")</f>
-        <v>4</v>
-      </c>
+      <c r="B48" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C48" s="38"/>
+      <c r="D48" s="39"/>
+      <c r="E48" s="16"/>
       <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5"/>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
-      <c r="K48" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="L48" s="19"/>
-      <c r="M48" s="16"/>
+      <c r="K48" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="L48" s="34"/>
+      <c r="M48" s="34"/>
       <c r="N48" s="5"/>
       <c r="O48" s="13" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="P48" s="13">
-        <v>14282</v>
+        <f>-C50</f>
+        <v>-15850</v>
       </c>
       <c r="Q48" s="5"/>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="5"/>
-      <c r="B49" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="C49" s="52">
-        <f>SUBTOTAL(9,C45:C48)</f>
-        <v>15925</v>
-      </c>
-      <c r="D49" s="53"/>
-      <c r="E49" s="21">
-        <f>E46</f>
-        <v>34</v>
-      </c>
+      <c r="B49" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="C49" s="40"/>
+      <c r="D49" s="41"/>
+      <c r="E49" s="25"/>
       <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
-      <c r="K49" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L49" s="23"/>
-      <c r="M49" s="23"/>
-      <c r="N49" s="5"/>
-      <c r="O49" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="P49" s="13">
-        <v>6005</v>
+      <c r="K49" s="35"/>
+      <c r="L49" s="36">
+        <f>SUBTOTAL(9,L44:L48)</f>
+        <v>1455</v>
+      </c>
+      <c r="M49" s="36">
+        <f>SUBTOTAL(9,M44:M48)</f>
+        <v>2</v>
+      </c>
+      <c r="O49" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="P49" s="3">
+        <f>SUBTOTAL(9,P44:P48)</f>
+        <v>17025</v>
       </c>
       <c r="Q49" s="5"/>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="5"/>
-      <c r="B50" s="32" t="s">
-        <v>41</v>
-      </c>
-      <c r="C50" s="38"/>
-      <c r="D50" s="39"/>
-      <c r="E50" s="16"/>
+      <c r="B50" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C50" s="42">
+        <f>C47+C48+C49</f>
+        <v>15850</v>
+      </c>
+      <c r="D50" s="43"/>
+      <c r="E50" s="27" t="s">
+        <v>47</v>
+      </c>
       <c r="F50" s="5"/>
-      <c r="I50" s="5"/>
+      <c r="G50" s="5"/>
       <c r="J50" s="5"/>
-      <c r="K50" s="33" t="s">
+      <c r="K50" s="5"/>
+      <c r="L50" s="37"/>
+      <c r="M50" s="37"/>
+      <c r="N50" s="37"/>
+      <c r="O50" s="5"/>
+      <c r="P50" s="5"/>
+      <c r="Q50" s="5"/>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K51" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L51" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M51" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K52" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="L52" s="12">
+        <f>SUMIFS(G$3:G$73,$J$3:$J$73,$K51)</f>
+        <v>3655</v>
+      </c>
+      <c r="M52" s="12">
+        <f>SUMIFS(Q3:Q73,J3:J73,K51)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K53" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="L53" s="12"/>
+      <c r="M53" s="16"/>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K54" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="L54" s="19"/>
+      <c r="M54" s="16"/>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K55" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="L55" s="23"/>
+      <c r="M55" s="23"/>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K56" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="L50" s="34"/>
-      <c r="M50" s="34"/>
-      <c r="N50" s="5"/>
-      <c r="O50" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="P50" s="13">
-        <f>-C52</f>
-        <v>-15925</v>
-      </c>
-      <c r="Q50" s="5"/>
-    </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A51" s="5"/>
-      <c r="B51" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="C51" s="40"/>
-      <c r="D51" s="41"/>
-      <c r="E51" s="25"/>
-      <c r="F51" s="5"/>
-      <c r="I51" s="5"/>
-      <c r="J51" s="5"/>
-      <c r="K51" s="35"/>
-      <c r="L51" s="36">
-        <f>SUBTOTAL(9,L46:L50)</f>
-        <v>1455</v>
-      </c>
-      <c r="M51" s="36">
-        <f>SUBTOTAL(9,M46:M50)</f>
-        <v>2</v>
-      </c>
-      <c r="O51" s="26" t="s">
-        <v>45</v>
-      </c>
-      <c r="P51" s="3">
-        <f>SUBTOTAL(9,P46:P50)</f>
-        <v>16950</v>
-      </c>
-      <c r="Q51" s="5"/>
-    </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A52" s="5"/>
-      <c r="B52" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C52" s="42">
-        <f>C49+C50+C51</f>
-        <v>15925</v>
-      </c>
-      <c r="D52" s="43"/>
-      <c r="E52" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
-      <c r="J52" s="5"/>
-      <c r="K52" s="5"/>
-      <c r="L52" s="37"/>
-      <c r="M52" s="37"/>
-      <c r="N52" s="37"/>
-      <c r="O52" s="5"/>
-      <c r="P52" s="5"/>
-      <c r="Q52" s="5"/>
-    </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K53" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="L53" s="7" t="s">
+      <c r="L56" s="34"/>
+      <c r="M56" s="34"/>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K57" s="35"/>
+      <c r="L57" s="36">
+        <f>SUBTOTAL(9,L52:L56)</f>
+        <v>3655</v>
+      </c>
+      <c r="M57" s="36">
+        <f>SUBTOTAL(9,M52:M56)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K59" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L59" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="M53" s="7" t="s">
+      <c r="M59" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K54" s="11" t="s">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K60" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L54" s="12">
-        <f>SUMIFS(G$3:G$75,$J$3:$J$75,$K53)</f>
-        <v>3655</v>
-      </c>
-      <c r="M54" s="12">
-        <f>SUMIFS(Q3:Q75,J3:J75,K53)</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K55" s="11" t="s">
+      <c r="L60" s="12">
+        <f>SUMIFS(G$3:G$73,$J$3:$J$73,$K59)</f>
+        <v>9555</v>
+      </c>
+      <c r="M60" s="12">
+        <f>SUMIFS(Q3:Q73,J3:J73,K59)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K61" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="L55" s="12"/>
-      <c r="M55" s="16"/>
-    </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K56" s="18" t="s">
+      <c r="L61" s="12"/>
+      <c r="M61" s="16"/>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K62" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L56" s="19"/>
-      <c r="M56" s="16"/>
-    </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K57" s="22" t="s">
+      <c r="L62" s="19"/>
+      <c r="M62" s="16"/>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K63" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="L57" s="23"/>
-      <c r="M57" s="23"/>
-    </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K58" s="33" t="s">
+      <c r="L63" s="23"/>
+      <c r="M63" s="23"/>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="K64" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="L58" s="34"/>
-      <c r="M58" s="34"/>
-    </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K59" s="35"/>
-      <c r="L59" s="36">
-        <f>SUBTOTAL(9,L54:L58)</f>
-        <v>3655</v>
-      </c>
-      <c r="M59" s="36">
-        <f>SUBTOTAL(9,M54:M58)</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K61" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="L61" s="7" t="s">
+      <c r="L64" s="34"/>
+      <c r="M64" s="34"/>
+    </row>
+    <row r="65" spans="11:13" x14ac:dyDescent="0.25">
+      <c r="K65" s="35"/>
+      <c r="L65" s="36">
+        <f>SUBTOTAL(9,L60:L64)</f>
+        <v>9555</v>
+      </c>
+      <c r="M65" s="36">
+        <f>SUBTOTAL(9,M60:M64)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67" spans="11:13" x14ac:dyDescent="0.25">
+      <c r="K67" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L67" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="M61" s="7" t="s">
+      <c r="M67" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K62" s="11" t="s">
+    <row r="68" spans="11:13" x14ac:dyDescent="0.25">
+      <c r="K68" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L62" s="12">
-        <f>SUMIFS(G$3:G$75,$J$3:$J$75,$K61)</f>
-        <v>9555</v>
-      </c>
-      <c r="M62" s="12">
-        <f>SUMIFS(Q3:Q75,J3:J75,K61)</f>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K63" s="11" t="s">
+      <c r="L68" s="12">
+        <f>SUMIFS(G$3:G$73,$J$3:$J$73,$K67)</f>
+        <v>5565</v>
+      </c>
+      <c r="M68" s="12">
+        <f>SUMIFS(Q3:Q73,J3:J73,K67)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="11:13" x14ac:dyDescent="0.25">
+      <c r="K69" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="L63" s="12"/>
-      <c r="M63" s="16"/>
-    </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="K64" s="18" t="s">
+      <c r="L69" s="12"/>
+      <c r="M69" s="16"/>
+    </row>
+    <row r="70" spans="11:13" x14ac:dyDescent="0.25">
+      <c r="K70" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="L64" s="19"/>
-      <c r="M64" s="16"/>
-    </row>
-    <row r="65" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K65" s="22" t="s">
+      <c r="L70" s="19"/>
+      <c r="M70" s="16"/>
+    </row>
+    <row r="71" spans="11:13" x14ac:dyDescent="0.25">
+      <c r="K71" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="L65" s="23"/>
-      <c r="M65" s="23"/>
-    </row>
-    <row r="66" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K66" s="33" t="s">
+      <c r="L71" s="23"/>
+      <c r="M71" s="23"/>
+    </row>
+    <row r="72" spans="11:13" x14ac:dyDescent="0.25">
+      <c r="K72" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="L66" s="34"/>
-      <c r="M66" s="34"/>
-    </row>
-    <row r="67" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K67" s="35"/>
-      <c r="L67" s="36">
-        <f>SUBTOTAL(9,L62:L66)</f>
-        <v>9555</v>
-      </c>
-      <c r="M67" s="36">
-        <f>SUBTOTAL(9,M62:M66)</f>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="69" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K69" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="L69" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="M69" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="70" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K70" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="L70" s="12">
-        <f>SUMIFS(G$3:G$75,$J$3:$J$75,$K69)</f>
+      <c r="L72" s="34"/>
+      <c r="M72" s="34"/>
+    </row>
+    <row r="73" spans="11:13" x14ac:dyDescent="0.25">
+      <c r="K73" s="35"/>
+      <c r="L73" s="36">
+        <f>SUBTOTAL(9,L68:L72)</f>
         <v>5565</v>
       </c>
-      <c r="M70" s="12">
-        <f>SUMIFS(Q3:Q75,J3:J75,K69)</f>
+      <c r="M73" s="36">
+        <f>SUBTOTAL(9,M68:M72)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K71" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="L71" s="12"/>
-      <c r="M71" s="16"/>
-    </row>
-    <row r="72" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K72" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="L72" s="19"/>
-      <c r="M72" s="16"/>
-    </row>
-    <row r="73" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K73" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="L73" s="23"/>
-      <c r="M73" s="23"/>
-    </row>
-    <row r="74" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K74" s="33" t="s">
-        <v>42</v>
-      </c>
-      <c r="L74" s="34"/>
-      <c r="M74" s="34"/>
-    </row>
-    <row r="75" spans="11:13" x14ac:dyDescent="0.25">
-      <c r="K75" s="35"/>
-      <c r="L75" s="36">
-        <f>SUBTOTAL(9,L70:L74)</f>
-        <v>5565</v>
-      </c>
-      <c r="M75" s="36">
-        <f>SUBTOTAL(9,M70:M74)</f>
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:Q66" xr:uid="{F28604F7-D21B-4533-8AD0-8E4BB48433FE}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:Q66">
-      <sortCondition ref="D2:D66"/>
+  <autoFilter ref="A2:Q64" xr:uid="{F28604F7-D21B-4533-8AD0-8E4BB48433FE}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:Q64">
+      <sortCondition ref="D2:D64"/>
     </sortState>
   </autoFilter>
   <mergeCells count="8">
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
     <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="C52:D52"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C44:D44"/>
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C49:D49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>